<commit_message>
Add REPO_CONVENTIONS.md + mark Mean Well NDR-480-24 as donated (/bin/bash)
REPO_CONVENTIONS.md documents the src/ subfolder pattern so AI
assistants and team members follow the same layout when adding
new content:
- folder/src/ = source files (xlsx, tex, py, images, project files)
- folder/    = rendered outputs (pdf) and standalone documents
                (vendor PDFs, signed contracts, markdown refs)

Includes a full current layout of the repo, rules for what goes
where, and what NOT to do.

BOM update: Mean Well NDR-480-24 24V power supply was donated to
the team (no cost). Unit cost set to $0 and description updated
to note this. Total cost in BOM header will recompute automatically.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="B1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -795,7 +795,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Mean Well 480 W, 24 VDC DIN-rail power supply for PLC, HMI, indicator LEDs, and VFD control loops.</t>
+          <t>Mean Well 480 W, 24 VDC DIN-rail power supply for PLC, HMI, indicator LEDs, and VFD control loops. Donated by sponsor / obtained at no cost to the EE team.</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="I13" s="7">
         <f>E13*H13</f>

</xml_diff>

<commit_message>
BOM: mark Phoenix TMC 8 3C 15A breaker as $0 (EPL free pile)
Phoenix Contact TMC 8 3C 15A circuit breaker (P/N 2907618) was
obtained at no cost from the PSU Electronics Prototyping Lab
free pile. Unit cost set to $0 and description updated.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -758,7 +758,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Phoenix Contact thermal-magnetic DIN-rail circuit breaker, 15 A, on VFD neutral leg (per as-built).</t>
+          <t>Phoenix Contact thermal-magnetic DIN-rail circuit breaker, 15 A, on VFD neutral leg (per as-built). Obtained at no cost from the PSU EPL free pile.</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="I12" s="7">
         <f>E12*H12</f>

</xml_diff>

<commit_message>
BOM: SD-N35 contactor actual cost $12.59 (per eBay receipt)
Mitsubishi SD-N35 magnetic contactor was purchased via eBay
seller tpmachinery (order 23-14145-39817, delivered Feb 2, 2026)
for $12.59 including shipping. BOM updated from the earlier
estimate of $35.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -845,11 +845,11 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/itm/186240xxxxxx</t>
+          <t>https://www.ebay.com/itm/... (tpmachinery seller, order 23-14145-39817, Jan 2026)</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>35</v>
+        <v>12.59</v>
       </c>
       <c r="I14" s="7">
         <f>E14*H14</f>

</xml_diff>

<commit_message>
BOM: PLC modules bundled as $350 used combo purchase (eBay)
Per eBay order 20-14113-87209 from seller planet-surplus
(delivered Jan 30 2026), the entire DL205 rack and module set
was purchased as a USED combo for $350 total:
  - D2-09B-1 chassis (DL205 9-slot base)
  - H2-DM1E CPU
  - D2-08ND3 discrete input
  - F2-08AD-1 analog current input
  - F2-04RTD RTD input
  - D2-08TR relay output (eBay listing said D2-08TD2; actual unit
    is D2-08TR which matches our build)
  - F2-08DA-2 analog voltage output (eBay listing said F2-02DA;
    actual unit is F2-08DA-2)
  - D2-FILL filler panels

Full $350 logged on the H2-DM1E row as the combo's anchor item.
All other PLC modules set to $0 with 'Included in the H2-DM1E
combo purchase' note in the description so the total cost stays
accurate without double-counting.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect Do-more CPU with built-in Ethernet, fits D2-09B-1 DL205 rack.</t>
+          <t>AutomationDirect Do-more CPU with built-in Ethernet, fits D2-09B-1 DL205 rack. Purchased Jan 2026 from planet-surplus as a USED combo for $350 total, includes: D2-09B-1 chassis, D2-08ND3, F2-08AD-1, F2-04RTD, D2-08TR, F2-08DA-2, and D2-FILL filler panels.</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
@@ -956,11 +956,11 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>https://www.automationdirect.com/</t>
+          <t>https://www.ebay.com/itm/... (planet-surplus seller, order 20-14113-87209, Jan 2026)</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>195</v>
+        <v>350</v>
       </c>
       <c r="I17" s="7">
         <f>E17*H17</f>
@@ -980,7 +980,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect DirectLOGIC 205 9-slot AC-powered base.</t>
+          <t>AutomationDirect DirectLOGIC 205 9-slot AC-powered base. Included in the H2-DM1E used combo purchase.</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="I18" s="7">
         <f>E18*H18</f>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect 8-ch, 24 VDC, sourcing/sinking discrete input module. Slot 2. Inputs X0-X7.</t>
+          <t>AutomationDirect 8-ch, 24 VDC, sourcing/sinking discrete input module. Slot 2. Inputs X0-X7. Included in the H2-DM1E used combo purchase.</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="H19" s="7" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="I19" s="7">
         <f>E19*H19</f>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect 8-ch, 4-20 mA analog current input module. Slot 3. CH1+ reads VFD VO current monitor.</t>
+          <t>AutomationDirect 8-ch, 4-20 mA analog current input module. Slot 3. CH1+ reads VFD VO current monitor. Included in the H2-DM1E used combo purchase.</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="I20" s="7">
         <f>E20*H20</f>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect 4-ch RTD input module. Slot 4. Installed but unused (spare).</t>
+          <t>AutomationDirect 4-ch RTD input module. Slot 4. Installed but unused (spare). Included in the H2-DM1E used combo purchase.</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>195</v>
+        <v>0</v>
       </c>
       <c r="I21" s="7">
         <f>E21*H21</f>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect 8-ch relay output module. Slot 5. Drives button LEDs (Y0-Y4) and VFD FOR/REV/RST (Y6/Y7/Y5).</t>
+          <t>AutomationDirect 8-ch relay output module. Slot 5. Drives button LEDs (Y0-Y4) and VFD FOR/REV/RST (Y6/Y7/Y5). Included in the H2-DM1E used combo purchase (eBay listing showed D2-08TD2 but seller substituted D2-08TR which is what we use).</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="I22" s="7">
         <f>E22*H22</f>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect 8-ch, 0-10 V analog voltage output module. Slot 6. +V1 drives VFD VI speed reference.</t>
+          <t>AutomationDirect 8-ch, 0-10 V analog voltage output module. Slot 6. +V1 drives VFD VI speed reference. Included in the H2-DM1E used combo purchase (eBay listing showed F2-02DA but actual unit is F2-08DA-2).</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>245</v>
+        <v>0</v>
       </c>
       <c r="I23" s="7">
         <f>E23*H23</f>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect blank fill panels for unused rack slots 7-9.</t>
+          <t>AutomationDirect blank fill panels for unused rack slots 7-9. Included in the H2-DM1E used combo purchase.</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I24" s="7">
         <f>E24*H24</f>

</xml_diff>

<commit_message>
BOM: banana sockets (blue/white/red) marked $0 (free pile)
All three motor-output banana sockets (U=blue, V=white, W=red)
obtained at no cost from a free pile. Unit costs set to $0 and
descriptions updated.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I49"/>
+  <dimension ref="B1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Generic 4 mm panel-mount banana socket, blue. Quick-disconnect for VFD U output to motor T1.</t>
+          <t>Generic 4 mm panel-mount banana socket, blue. Quick-disconnect for VFD U output to motor T1. Obtained at no cost from a free pile.</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr"/>
       <c r="H37" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I37" s="7">
         <f>E37*H37</f>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Generic 4 mm panel-mount banana socket, white. VFD V output to motor T2.</t>
+          <t>Generic 4 mm panel-mount banana socket, white. VFD V output to motor T2. Obtained at no cost from a free pile.</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G38" s="5" t="inlineStr"/>
       <c r="H38" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I38" s="7">
         <f>E38*H38</f>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Generic 4 mm panel-mount banana socket, red. VFD W output to motor T3.</t>
+          <t>Generic 4 mm panel-mount banana socket, red. VFD W output to motor T3. Obtained at no cost from a free pile.</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr"/>
       <c r="H39" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I39" s="7">
         <f>E39*H39</f>
@@ -2094,6 +2094,16 @@
         <v/>
       </c>
     </row>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BOM: V30AE000055 ferrules moved from Combined to Excluded
Z+F V30AE000055 12 AWG ferrules were purchased from URS Electronics
but ultimately not used in the as-built panel. Removed from the
Combined BOM and added to the Excluded - Not Used sheet with reason
'Purchased but not used; spare stock retained'.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I59"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1846,50 +1846,50 @@
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>V30AE000055</t>
+          <t>18 AWG Blue</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Insulated Ferrules, 12 AWG</t>
+          <t>Control Wire, Blue</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Z+F crimp ferrules, 12 AWG, 10 mm length, gray (DIN color code). 500-piece pack.</t>
+          <t>18 AWG stranded blue control wire (NFPA 79 §13.2 DC control).</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>Roll</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
       <c r="H42" s="7" t="n">
-        <v>0.023</v>
+        <v>25</v>
       </c>
       <c r="I42" s="7">
-        <f>E42*H42</f>
+        <f>E43*H43</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>18 AWG Blue</t>
+          <t>18 AWG White</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Control Wire, Blue</t>
+          <t>Control Return Wire</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>18 AWG stranded blue control wire (NFPA 79 §13.2 DC control).</t>
+          <t>18 AWG stranded white wire for DC return (NFPA 79 §13.2).</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
@@ -1902,27 +1902,27 @@
       </c>
       <c r="G43" s="5" t="inlineStr"/>
       <c r="H43" s="7" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I43" s="7">
-        <f>E43*H43</f>
+        <f>E44*H44</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>18 AWG White</t>
+          <t>12 AWG Black</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Control Return Wire</t>
+          <t>Power Wire, Black</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>18 AWG stranded white wire for DC return (NFPA 79 §13.2).</t>
+          <t>12 AWG black wire for AC mains and motor leads.</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
@@ -1935,27 +1935,27 @@
       </c>
       <c r="G44" s="5" t="inlineStr"/>
       <c r="H44" s="7" t="n">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="I44" s="7">
-        <f>E44*H44</f>
+        <f>E45*H45</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>12 AWG Black</t>
+          <t>12 AWG Green/Yellow</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Power Wire, Black</t>
+          <t>Ground Wire</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>12 AWG black wire for AC mains and motor leads.</t>
+          <t>12 AWG green/yellow stranded equipment grounding wire (NFPA 79).</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
@@ -1968,27 +1968,27 @@
       </c>
       <c r="G45" s="5" t="inlineStr"/>
       <c r="H45" s="7" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="I45" s="7">
-        <f>E45*H45</f>
+        <f>E46*H46</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>12 AWG Green/Yellow</t>
+          <t>GMA-500mA or 0217.500MXP</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Ground Wire</t>
+          <t>Fuse - 500 mA F</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>12 AWG green/yellow stranded equipment grounding wire (NFPA 79).</t>
+          <t>Bussmann or Littelfuse 5x20 mm fast-blow fuse, 500 mA, 250 V. (Currently not installed per as-built note - retained as recommended addition.)</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
@@ -1996,32 +1996,32 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>Roll</t>
+          <t>EA</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
       <c r="H46" s="7" t="n">
-        <v>40</v>
+        <v>1.5</v>
       </c>
       <c r="I46" s="7">
-        <f>E46*H46</f>
+        <f>E47*H47</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>GMA-500mA or 0217.500MXP</t>
+          <t>GMA-1A or equiv.</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Fuse - 500 mA F</t>
+          <t>Fuse - 1 A F</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Bussmann or Littelfuse 5x20 mm fast-blow fuse, 500 mA, 250 V. (Currently not installed per as-built note - retained as recommended addition.)</t>
+          <t>5x20 mm fast-blow fuse, 1 A, 250 V. Protects shared +24 V pushbutton common (in EURO S4LH).</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
@@ -2037,73 +2037,30 @@
         <v>1.5</v>
       </c>
       <c r="I47" s="7">
-        <f>E47*H47</f>
+        <f>E48*H48</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>GMA-1A or equiv.</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Fuse - 1 A F</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>5x20 mm fast-blow fuse, 1 A, 250 V. Protects shared +24 V pushbutton common (in EURO S4LH).</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr"/>
-      <c r="H48" s="7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I48" s="7">
-        <f>E48*H48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="D49" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>TOTAL PARTS</t>
         </is>
       </c>
-      <c r="E49" s="2">
+      <c r="E48" s="2">
         <f>SUM(E8:E48)</f>
         <v/>
       </c>
-      <c r="G49" s="8" t="inlineStr">
+      <c r="G48" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="I49" s="3">
+      <c r="I48" s="3">
         <f>SUM(I8:I48)</f>
         <v/>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -2117,7 +2074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2721,6 +2678,33 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>V30AE000055</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Insulated Ferrules, 12 AWG (gray)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Z+F crimp ferrules, 12 AWG, 10 mm length, gray (DIN color code). 500-piece pack.</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>URS Electronics invoice (purchased but not used)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Purchased from URS Electronics but ultimately not used in the as-built panel. Spare stock retained for future projects.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BOM: all control and power wires marked $0 (free / existing stock)
18 AWG Blue, 18 AWG White, 12 AWG Black, and 12 AWG Green/Yellow
wires obtained at no cost - some from team member existing home
stock, some from the free pile. Cost set to $0 and descriptions
updated.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="B1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>18 AWG stranded blue control wire (NFPA 79 §13.2 DC control).</t>
+          <t>18 AWG stranded blue control wire (NFPA 79 §13.2 DC control). Obtained at no cost (some from team member's existing stock, some from free pile).</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr"/>
       <c r="H42" s="7" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I42" s="7">
         <f>E43*H43</f>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>18 AWG stranded white wire for DC return (NFPA 79 §13.2).</t>
+          <t>18 AWG stranded white wire for DC return (NFPA 79 §13.2). Obtained at no cost (some from team member's existing stock, some from free pile).</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr"/>
       <c r="H43" s="7" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="I43" s="7">
         <f>E44*H44</f>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>12 AWG black wire for AC mains and motor leads.</t>
+          <t>12 AWG black wire for AC mains and motor leads. Obtained at no cost (some from team member's existing stock, some from free pile).</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr"/>
       <c r="H44" s="7" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I44" s="7">
         <f>E45*H45</f>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>12 AWG green/yellow stranded equipment grounding wire (NFPA 79).</t>
+          <t>12 AWG green/yellow stranded equipment grounding wire (NFPA 79). Obtained at no cost (some from team member's existing stock, some from free pile).</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr"/>
       <c r="H45" s="7" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I45" s="7">
         <f>E46*H46</f>
@@ -2061,6 +2061,17 @@
         <v/>
       </c>
     </row>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BOM: fix AMOUNT, PART COUNT, and TOTAL COST formulas
After earlier row deletions, the SUM ranges in the header and
totals row included the totals row itself (E8:E48 covering row 48
which IS the totals row), causing recursive/erroneous totals.
Also the last data row's AMOUNT formula was pointing at the totals
row instead of its own row.

Rebuilt all formulas:
- Every data row's AMOUNT (col I) now correctly = E<row>*H<row>
- TOTAL row sums only the actual data range (8 to last data row)
- Header PART COUNT and TOTAL COST use the same correct range

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I59"/>
+  <dimension ref="B1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="C4" s="2">
-        <f>SUM(E8:E48)</f>
+        <f>SUM(E8:E47)</f>
         <v/>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>SUM(I8:I48)</f>
+        <f>SUM(I8:I47)</f>
         <v/>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -1872,7 +1872,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="7">
-        <f>E43*H43</f>
+        <f>E42*H42</f>
         <v/>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="7">
-        <f>E44*H44</f>
+        <f>E43*H43</f>
         <v/>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
         <v>0</v>
       </c>
       <c r="I44" s="7">
-        <f>E45*H45</f>
+        <f>E44*H44</f>
         <v/>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="7">
-        <f>E46*H46</f>
+        <f>E45*H45</f>
         <v/>
       </c>
     </row>
@@ -2004,7 +2004,7 @@
         <v>1.5</v>
       </c>
       <c r="I46" s="7">
-        <f>E47*H47</f>
+        <f>E46*H46</f>
         <v/>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
         <v>1.5</v>
       </c>
       <c r="I47" s="7">
-        <f>E48*H48</f>
+        <f>E47*H47</f>
         <v/>
       </c>
     </row>
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E48" s="2">
-        <f>SUM(E8:E48)</f>
+        <f>SUM(E8:E47)</f>
         <v/>
       </c>
       <c r="G48" s="8" t="inlineStr">
@@ -2057,21 +2057,10 @@
         </is>
       </c>
       <c r="I48" s="3">
-        <f>SUM(I8:I48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
+        <f>SUM(I8:I47)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BOM: brake resistor now LS Electric APCS-300R30-AD from AutomationDirect ($29)
Original ATO-branded APCS-300R30-AD was ordered but never arrived
after shipping. Replaced with the LS Electric APCS-300R30-AD (same
part number / specifications) purchased from AutomationDirect for
$29. Updated manufacturer, unit cost, link, and description.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -684,7 +684,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>ATO 300 W, 30 ohm aluminum-clad braking resistor for VFD dynamic braking on P+/PR.</t>
+          <t>LS Electric 300 W, 30 ohm aluminum-clad braking resistor for VFD dynamic braking on P+/PR. Purchased from AutomationDirect. Note: an earlier identical-part-number unit (ATO branded) was ordered but never arrived after shipping; replaced with this LS Electric unit which is the brake resistor actually installed.</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
@@ -697,11 +697,11 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>https://www.ato.com/</t>
+          <t>https://www.automationdirect.com/adc/shopping/catalog/motion_control/ls_electric_l7c_(l7ca_series)_servo_systems/servo_accessories/apcs-300r30-ad</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="I10" s="7">
         <f>E10*H10</f>

</xml_diff>

<commit_message>
BOM: add Seloky LM2596 DC-DC buck converter for capacitive touch module
Adds Seloky LM2596 adjustable DC-DC buck converter (2-pack with
voltmeter display) sourced from Amazon for $7.99. Steps down the
24 VDC panel supply to the input voltage required by the
capacitive touch module sub-circuit.

Formulas rebuilt to extend the data range through the new row.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -97,6 +97,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -529,7 +530,7 @@
         </is>
       </c>
       <c r="C4" s="2">
-        <f>SUM(E8:E47)</f>
+        <f>SUM(E8:E48)</f>
         <v/>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -545,7 +546,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>SUM(I8:I47)</f>
+        <f>SUM(I8:I48)</f>
         <v/>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -2042,22 +2043,60 @@
       </c>
     </row>
     <row r="48">
-      <c r="D48" s="8" t="inlineStr">
+      <c r="A48" s="9" t="inlineStr"/>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>LM2596</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>DC-DC Buck Converter (24V to 5V/3.3V)</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Seloky LM2596-based adjustable DC-DC buck converter module with voltmeter display (sold as 2-pack). Steps down 24 VDC panel supply to the input voltage required by the capacitive touch module.</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/Converter-Adjustable-Regulator-Voltmeter-Display/dp/B0F1M2SR31</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="I48" s="7">
+        <f>E48*H48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>TOTAL PARTS</t>
         </is>
       </c>
-      <c r="E48" s="2">
-        <f>SUM(E8:E47)</f>
-        <v/>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
+      <c r="E49" s="2">
+        <f>SUM(E8:E48)</f>
+        <v/>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="I48" s="3">
-        <f>SUM(I8:I47)</f>
+      <c r="I49" s="3">
+        <f>SUM(I8:I48)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BOM: HMI actual cost $148.95, add enclosure and 3V relay
Three updates:
- HMI EA1-T4CL: actual eBay purchase cost set to $148.95 (was $125
  estimate). Link updated to the actual auction. The unit was
  purchased used and included the serial cable.
- New: Vorksmen SEB001 control panel enclosure ($59.98). Houses
  the entire electrical system.
- New: AEDIKO AE14921a 3 VDC PCB-mount relay ($6.99). Used in the
  capacitive touch module sub-circuit to interface the low-voltage
  touch output with the 24 VDC panel control voltage.

All AMOUNT, SUM, and header formulas rebuilt for the new row range.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/src/BOM_Combined_As_Built.xlsx
+++ b/BOM/src/BOM_Combined_As_Built.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="C4" s="2">
-        <f>SUM(E8:E48)</f>
+        <f>SUM(E8:E50)</f>
         <v/>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>SUM(I8:I48)</f>
+        <f>SUM(I8:I50)</f>
         <v/>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>AutomationDirect C-More Micro-Graphic 4-inch color touch panel HMI. Purchase included the serial cable for HMI-to-CPU communication (RS-232 to H2-DM1E serial port).</t>
+          <t>AutomationDirect C-More Micro-Graphic 4-inch color touch panel HMI. Purchased used from eBay for $148.95 (Apr 2026). Purchase included the serial cable for HMI-to-CPU communication (RS-232 to H2-DM1E serial port).</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
@@ -1253,11 +1253,11 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/itm/306660xxxxxx</t>
+          <t>https://www.ebay.com/itm/306662618920</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>125</v>
+        <v>148.95</v>
       </c>
       <c r="I25" s="7">
         <f>E25*H25</f>
@@ -2081,22 +2081,96 @@
       </c>
     </row>
     <row r="49">
-      <c r="D49" s="8" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>SEB001</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Control Panel Enclosure</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Vorksmen industrial control enclosure (steel) housing the entire electrical system including PLC rack, VFD, contactor, PSU, terminal blocks, and operator panel.</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="n">
+        <v>59.98</v>
+      </c>
+      <c r="I49" s="7">
+        <f>E49*H49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>AE14921a</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>3V Relay</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>AEDIKO 3 VDC PCB-mount relay. Used in the capacitive touch module sub-circuit to interface the low-voltage touch sensor output with the 24 VDC panel control voltage.</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="I50" s="7">
+        <f>E50*H50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="D51" s="8" t="inlineStr">
         <is>
           <t>TOTAL PARTS</t>
         </is>
       </c>
-      <c r="E49" s="2">
-        <f>SUM(E8:E48)</f>
-        <v/>
-      </c>
-      <c r="G49" s="8" t="inlineStr">
+      <c r="E51" s="2">
+        <f>SUM(E8:E50)</f>
+        <v/>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="I49" s="3">
-        <f>SUM(I8:I48)</f>
+      <c r="I51" s="3">
+        <f>SUM(I8:I50)</f>
         <v/>
       </c>
     </row>

</xml_diff>